<commit_message>
Update investment costs for different interest rates
</commit_message>
<xml_diff>
--- a/data/Berechnungen.xlsx
+++ b/data/Berechnungen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\2.b_Hybrider_Netzzugang\1_Model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\LEGO-Pyomo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EB843E-864A-4DF7-9084-019B65252DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8CE4C5E-8503-4F50-A69E-1FC986F49E08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35980" yWindow="3350" windowWidth="28490" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="570" yWindow="4730" windowWidth="28800" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CAPEX" sheetId="1" r:id="rId1"/>
@@ -32,12 +32,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
   <si>
     <t>PV Investment Kosten 2025 [€/MW]</t>
   </si>
@@ -64,9 +67,6 @@
   </si>
   <si>
     <t>Sources</t>
-  </si>
-  <si>
-    <t>https://www.ise.fraunhofer.de/en/publications/studies/cost-of-electricity.html</t>
   </si>
   <si>
     <t>A comprehensive review of CAPEX-driven LCOE optimization strategies for utility-scale PV systems; Dhanup et al.</t>
@@ -179,6 +179,30 @@
   </si>
   <si>
     <t>5 % Interest</t>
+  </si>
+  <si>
+    <t>https://www.irena.org/-/media/Files/IRENA/Agency/Publication/2026/Jul/IRENA_TEC_RPGC_in_2025_2026.pdf</t>
+  </si>
+  <si>
+    <t>für 2025</t>
+  </si>
+  <si>
+    <t>https://www.energy-storage.news/battery-storage-system-prices-continue-to-fall-sharply-bnef-and-ember-reports-find/</t>
+  </si>
+  <si>
+    <t>für 2035</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>NREL- Cost projection for utility scale Battery Storage:2025 Update</t>
+  </si>
+  <si>
+    <t>PV/Storage</t>
+  </si>
+  <si>
+    <t>Storage Range 2035 160-210€/MWh</t>
   </si>
 </sst>
 </file>
@@ -230,11 +254,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -515,46 +540,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:M38"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="38.3515625" customWidth="1"/>
-    <col min="3" max="3" width="10.29296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.36328125" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B1" s="4">
+        <v>667000</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
-        <v>620000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B2" s="4">
+        <v>520000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4">
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>19</v>
       </c>
-      <c r="B3">
-        <v>450000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.5">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4">
-        <v>320000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="B4" s="4">
+        <v>160000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -562,28 +587,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6">
         <f>0.02*B3</f>
-        <v>9000</v>
+        <v>4400</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.5">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7">
         <f>0.02*B4</f>
-        <v>6400</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.5">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -591,7 +616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -599,7 +624,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -607,7 +632,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -615,7 +640,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -626,89 +651,120 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
         <v>28</v>
       </c>
-      <c r="C14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.5">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" s="2">
         <f>($B1+$B$5)*(B$12*(1+B$12)^$B$10)/((1+B$12)^$B$10-1)</f>
-        <v>4082.8672463625344</v>
+        <v>34031.172467350807</v>
       </c>
       <c r="C15" s="2">
         <f>($B1+$B$5)*(C$12*(1+C$12)^$B$10)/((1+C$12)^$B$10-1)</f>
-        <v>5205.8061437342139</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.5">
+        <v>43390.998535856568</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" s="2">
         <f>($B2+$B$5)*(B$12*(1+B$12)^$B$10)/((1+B$12)^$B$10-1)</f>
-        <v>31633.267279298936</v>
+        <v>26531.341347273676</v>
       </c>
       <c r="C16" s="2">
         <f>($B2+$B$5)*(C$12*(1+C$12)^$B$10)/((1+C$12)^$B$10-1)</f>
-        <v>40333.58108708357</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
+        <v>33828.437579055906</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" s="2">
         <f>($B3+B6)*(B$12*(1+B$12)^$B$11)/((1+B$12)^$B$11-1)</f>
-        <v>38448.860432190217</v>
+        <v>18797.220655737441</v>
       </c>
       <c r="C17" s="2">
         <f>($B3+C6)*(C$12*(1+C$12)^$B$11)/((1+C$12)^$B$11-1)</f>
-        <v>43354.029424159962</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.5">
+        <v>21195.303274033755</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18" s="2">
         <f>($B4+B7)*(B$12*(1+B$12)^$B$11)/((1+B$12)^$B$11-1)</f>
-        <v>27341.411862890822</v>
+        <v>13670.705931445411</v>
       </c>
       <c r="C18" s="2">
         <f>($B4+C7)*(C$12*(1+C$12)^$B$11)/((1+C$12)^$B$11-1)</f>
-        <v>30829.532034958196</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
+        <v>15414.766017479098</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>29</v>
+      </c>
+      <c r="J33" t="s">
+        <v>30</v>
+      </c>
+      <c r="K33" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J34" t="s">
+        <v>32</v>
+      </c>
+      <c r="K34" t="s">
+        <v>33</v>
+      </c>
+      <c r="M34" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="J35" t="s">
+        <v>32</v>
+      </c>
+      <c r="K35" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A34" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A35" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A36" t="s">
-        <v>22</v>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -719,22 +775,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44C987FF-1052-4543-AB50-0C32197CACBC}">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>0.89500000000000002</v>
@@ -743,9 +799,9 @@
         <v>0.92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>0.92</v>
@@ -754,9 +810,9 @@
         <v>0.93500000000000005</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <f>B2*B3</f>
@@ -767,7 +823,7 @@
         <v>0.86020000000000008</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>2025</v>
       </c>
@@ -775,14 +831,14 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A29" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>